<commit_message>
Clean up import process to include Business Resource Code ID
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/LaborTypesAndSpread.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/LaborTypesAndSpread.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="18625"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twilson3\tfs\genBOE\dev\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e403038\source\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51B39803-94A5-47AD-A734-3BCB1316003D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="90" windowWidth="19320" windowHeight="11760"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Labor Types" sheetId="3" r:id="rId1"/>
@@ -91,7 +92,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/yyyy"/>
   </numFmts>
@@ -174,7 +175,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="genBOE" xfId="1"/>
+    <cellStyle name="genBOE" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -191,9 +192,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -231,9 +232,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -266,26 +267,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -318,26 +302,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -510,27 +477,27 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BZ2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.140625" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="30.7109375" customWidth="1"/>
-    <col min="3" max="3" width="30.28515625" customWidth="1"/>
-    <col min="4" max="4" width="31.28515625" customWidth="1"/>
-    <col min="5" max="5" width="30.42578125" customWidth="1"/>
-    <col min="6" max="6" width="30.85546875" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" customWidth="1"/>
-    <col min="8" max="8" width="15.28515625" customWidth="1"/>
-    <col min="9" max="9" width="15.140625" customWidth="1"/>
-    <col min="10" max="10" width="15.7109375" customWidth="1"/>
-    <col min="11" max="11" width="13.42578125" customWidth="1"/>
-    <col min="12" max="12" width="15.7109375" customWidth="1"/>
-    <col min="13" max="13" width="16.7109375" customWidth="1"/>
-    <col min="14" max="49" width="11.5703125" customWidth="1"/>
+    <col min="1" max="1" width="9.1796875" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="30.7265625" customWidth="1"/>
+    <col min="3" max="3" width="30.26953125" customWidth="1"/>
+    <col min="4" max="4" width="31.26953125" customWidth="1"/>
+    <col min="5" max="5" width="30.453125" customWidth="1"/>
+    <col min="6" max="6" width="30.81640625" customWidth="1"/>
+    <col min="7" max="7" width="12.453125" customWidth="1"/>
+    <col min="8" max="8" width="15.26953125" customWidth="1"/>
+    <col min="9" max="9" width="15.1796875" customWidth="1"/>
+    <col min="10" max="10" width="15.7265625" customWidth="1"/>
+    <col min="11" max="11" width="13.453125" customWidth="1"/>
+    <col min="12" max="12" width="15.7265625" customWidth="1"/>
+    <col min="13" max="13" width="16.7265625" customWidth="1"/>
+    <col min="14" max="49" width="11.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:78" s="4" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:78" s="4" customFormat="1" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="4" t="s">
         <v>7</v>
       </c>
@@ -766,7 +733,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:78" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:78" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
       <c r="M2" s="5"/>
@@ -775,18 +742,22 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="3" width="30.7109375" customWidth="1"/>
+    <col min="1" max="3" width="30.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>6</v>
       </c>
@@ -806,12 +777,16 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="C2" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -919,6 +894,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
   <documentManagement>
     <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
@@ -929,15 +913,6 @@
     </SipLabel>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -960,6 +935,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE4C072F-EAF4-499E-9347-564ED0FAEA38}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE9C6564-CDD5-499C-B8DC-E1612B398E0A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -974,12 +957,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE4C072F-EAF4-499E-9347-564ED0FAEA38}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>